<commit_message>
Navratnost 30 a 100 tipov
</commit_message>
<xml_diff>
--- a/public/TipRadar-navratnost-clenstva.xlsx
+++ b/public/TipRadar-navratnost-clenstva.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pásmo 65-80 %" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pásmo 68-80 %" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="65-80 % · 30 tipov" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="65-80 % · 100 tipov" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="68-80 % · 30 tipov" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="68-80 % · 100 tipov" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +579,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>
@@ -1419,7 +1421,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TipRadar – návratnosť členstva · pásmo 68 – 80 %</t>
+          <t>TipRadar – návratnosť členstva · pásmo 65 – 80 %</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1473,7 +1475,1799 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>60</v>
+        <v>100</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Model mieri na (úspešnosť)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Kurzy (môžete zmeniť)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Bez členstva (len vklady)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Potrebná úspešnosť</t>
+        </is>
+      </c>
+      <c r="B11" s="10">
+        <f>1/B$8</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>1/C$8</f>
+        <v/>
+      </c>
+      <c r="D11" s="10">
+        <f>1/D$8</f>
+        <v/>
+      </c>
+      <c r="E11" s="10">
+        <f>1/E$8</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Silver – 1 mesiac (49 €)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C13" s="11">
+        <f>49/1</f>
+        <v/>
+      </c>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B14" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C14" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D14" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E14" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Gold – 3 mesiace (119 €)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C20" s="11">
+        <f>119/3</f>
+        <v/>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B21" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C21" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D21" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E21" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Platinum – 6 mesiacov (219 €)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C27" s="11">
+        <f>219/6</f>
+        <v/>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B28" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C28" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D28" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E28" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Zelená = aspoň 3 body pod cieľom modelu · žltá = tesne pod ním · červená = nad ním (náročné).</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Vzorec: (1 + mesačná cena ÷ (počet tipov × vklad)) ÷ kurz</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Výpočet ukazuje len hranicu návratnosti, výhru nezaručuje. 18+</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B11:E34">
+    <cfRule type="cellIs" priority="1" operator="lessThanOrEqual" dxfId="0">
+      <formula>$B$6-0.03</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>$B$6-0.03</formula>
+      <formula>$B$6</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
+      <formula>$B$6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TipRadar – návratnosť členstva · pásmo 68 – 80 %</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Priemerná mesačná úspešnosť, pri ktorej sa vrátia vklady aj cena členstva. Zvýraznené políčka (bank, počet tipov, cieľ, kurzy) môžete zmeniť.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bank (€)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tipov mesačne</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Model mieri na (úspešnosť)</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Kurzy (môžete zmeniť)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="n"/>
+      <c r="G9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Bez členstva (len vklady)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Potrebná úspešnosť</t>
+        </is>
+      </c>
+      <c r="B11" s="10">
+        <f>1/B$8</f>
+        <v/>
+      </c>
+      <c r="C11" s="10">
+        <f>1/C$8</f>
+        <v/>
+      </c>
+      <c r="D11" s="10">
+        <f>1/D$8</f>
+        <v/>
+      </c>
+      <c r="E11" s="10">
+        <f>1/E$8</f>
+        <v/>
+      </c>
+      <c r="F11" s="2" t="n"/>
+      <c r="G11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Silver – 1 mesiac (49 €)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C13" s="11">
+        <f>49/1</f>
+        <v/>
+      </c>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B14" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C14" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D14" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E14" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E16" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E17" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>(1+$C$13/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Gold – 3 mesiace (119 €)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C20" s="11">
+        <f>119/3</f>
+        <v/>
+      </c>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B21" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C21" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D21" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E21" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E22" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E23" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F23" s="2" t="n"/>
+      <c r="G23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E24" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E25" s="10">
+        <f>(1+$C$20/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
+      <c r="G26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Platinum – 6 mesiacov (219 €)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>cena mesačne</t>
+        </is>
+      </c>
+      <c r="C27" s="11">
+        <f>219/6</f>
+        <v/>
+      </c>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Vklad na tip</t>
+        </is>
+      </c>
+      <c r="B28" s="13">
+        <f>"kurz "&amp;TEXT(B$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="C28" s="13">
+        <f>"kurz "&amp;TEXT(C$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="D28" s="13">
+        <f>"kurz "&amp;TEXT(D$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="E28" s="13">
+        <f>"kurz "&amp;TEXT(E$8,"0.00")</f>
+        <v/>
+      </c>
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <f>"1 % ("&amp;TEXT($B$4*0.01,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/B$8</f>
+        <v/>
+      </c>
+      <c r="C29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/C$8</f>
+        <v/>
+      </c>
+      <c r="D29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/D$8</f>
+        <v/>
+      </c>
+      <c r="E29" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.01))/E$8</f>
+        <v/>
+      </c>
+      <c r="F29" s="2" t="n"/>
+      <c r="G29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2">
+        <f>"2 % ("&amp;TEXT($B$4*0.02,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/B$8</f>
+        <v/>
+      </c>
+      <c r="C30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/C$8</f>
+        <v/>
+      </c>
+      <c r="D30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/D$8</f>
+        <v/>
+      </c>
+      <c r="E30" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.02))/E$8</f>
+        <v/>
+      </c>
+      <c r="F30" s="2" t="n"/>
+      <c r="G30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <f>"3 % ("&amp;TEXT($B$4*0.03,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/B$8</f>
+        <v/>
+      </c>
+      <c r="C31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/C$8</f>
+        <v/>
+      </c>
+      <c r="D31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/D$8</f>
+        <v/>
+      </c>
+      <c r="E31" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.03))/E$8</f>
+        <v/>
+      </c>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <f>"5 % ("&amp;TEXT($B$4*0.05,"0")&amp;" €)"</f>
+        <v/>
+      </c>
+      <c r="B32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/B$8</f>
+        <v/>
+      </c>
+      <c r="C32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/C$8</f>
+        <v/>
+      </c>
+      <c r="D32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/D$8</f>
+        <v/>
+      </c>
+      <c r="E32" s="10">
+        <f>(1+$C$27/($B$5*$B$4*0.05))/E$8</f>
+        <v/>
+      </c>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Zelená = aspoň 3 body pod cieľom modelu · žltá = tesne pod ním · červená = nad ním (náročné).</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Vzorec: (1 + mesačná cena ÷ (počet tipov × vklad)) ÷ kurz</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Výpočet ukazuje len hranicu návratnosti, výhru nezaručuje. 18+</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+      <c r="E37" s="2" t="n"/>
+      <c r="F37" s="2" t="n"/>
+      <c r="G37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+      <c r="E38" s="2" t="n"/>
+      <c r="F38" s="2" t="n"/>
+      <c r="G38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+      <c r="E39" s="2" t="n"/>
+      <c r="F39" s="2" t="n"/>
+      <c r="G39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+      <c r="E40" s="2" t="n"/>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+      <c r="E41" s="2" t="n"/>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+      <c r="E42" s="2" t="n"/>
+      <c r="F42" s="2" t="n"/>
+      <c r="G42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+      <c r="E44" s="2" t="n"/>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="2" t="n"/>
+      <c r="F45" s="2" t="n"/>
+      <c r="G45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="n"/>
+      <c r="G46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+      <c r="E47" s="2" t="n"/>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="2" t="n"/>
+      <c r="F48" s="2" t="n"/>
+      <c r="G48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+      <c r="E49" s="2" t="n"/>
+      <c r="F49" s="2" t="n"/>
+      <c r="G49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+      <c r="E50" s="2" t="n"/>
+      <c r="F50" s="2" t="n"/>
+      <c r="G50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+      <c r="E51" s="2" t="n"/>
+      <c r="F51" s="2" t="n"/>
+      <c r="G51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+      <c r="E52" s="2" t="n"/>
+      <c r="F52" s="2" t="n"/>
+      <c r="G52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+      <c r="E53" s="2" t="n"/>
+      <c r="F53" s="2" t="n"/>
+      <c r="G53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+      <c r="E54" s="2" t="n"/>
+      <c r="F54" s="2" t="n"/>
+      <c r="G54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+      <c r="E55" s="2" t="n"/>
+      <c r="F55" s="2" t="n"/>
+      <c r="G55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+      <c r="E56" s="2" t="n"/>
+      <c r="F56" s="2" t="n"/>
+      <c r="G56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+      <c r="E57" s="2" t="n"/>
+      <c r="F57" s="2" t="n"/>
+      <c r="G57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="n"/>
+      <c r="F58" s="2" t="n"/>
+      <c r="G58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="n"/>
+      <c r="F59" s="2" t="n"/>
+      <c r="G59" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="B11:E34">
+    <cfRule type="cellIs" priority="1" operator="lessThanOrEqual" dxfId="0">
+      <formula>$B$6-0.03</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>$B$6-0.03</formula>
+      <formula>$B$6</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
+      <formula>$B$6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TipRadar – návratnosť členstva · pásmo 68 – 80 %</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Priemerná mesačná úspešnosť, pri ktorej sa vrátia vklady aj cena členstva. Zvýraznené políčka (bank, počet tipov, cieľ, kurzy) môžete zmeniť.</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bank (€)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Tipov mesačne</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>100</v>
       </c>
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="n"/>

</xml_diff>

<commit_message>
Navratnost kalkulacka s vlastnym bankom
</commit_message>
<xml_diff>
--- a/public/TipRadar-navratnost-clenstva.xlsx
+++ b/public/TipRadar-navratnost-clenstva.xlsx
@@ -192,7 +192,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -295,11 +295,40 @@
         <color rgb="002E2E34"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00C9A55C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00C9A55C"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C9A55C"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00C9A55C"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -396,6 +425,14 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="14" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -868,7 +905,7 @@
       <c r="A5" s="1" t="n"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Priemerná mesačná úspešnosť, pri ktorej sa vrátia vklady aj cena členstva. Pod percentom: koľko tipov musí vyjsť z mesiaca a zo 100 tipov. Zlaté políčka môžete prepísať.</t>
+          <t>Priemerná mesačná úspešnosť, pri ktorej sa vrátia vklady aj cena členstva. Pod percentom: koľko tipov musí vyjsť za mesiac a koľko zo 100 tipov celkovo (nie mesačne). Zlaté políčka (bank, počet tipov, cieľ, kurzy) môžete prepísať – napr. bank 200 €.</t>
         </is>
       </c>
       <c r="H5" s="1" t="n"/>
@@ -1083,12 +1120,12 @@
       <c r="C16" s="14" t="n"/>
       <c r="D16" s="14" t="n"/>
       <c r="E16" s="14" t="n"/>
-      <c r="F16" s="22" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>49 €</t>
         </is>
       </c>
-      <c r="G16" s="23" t="n"/>
+      <c r="G16" s="41" t="n"/>
       <c r="H16" s="1" t="n"/>
       <c r="I16" s="1" t="n"/>
       <c r="J16" s="1" t="n"/>
@@ -1104,11 +1141,11 @@
       <c r="C17" s="24" t="n"/>
       <c r="D17" s="24" t="n"/>
       <c r="E17" s="24" t="n"/>
-      <c r="F17" s="25">
+      <c r="F17" s="42">
         <f>49/1</f>
         <v/>
       </c>
-      <c r="G17" s="26" t="n"/>
+      <c r="G17" s="43" t="n"/>
       <c r="H17" s="1" t="n"/>
       <c r="I17" s="1" t="n"/>
       <c r="J17" s="1" t="n"/>
@@ -1153,23 +1190,23 @@
         <v/>
       </c>
       <c r="C19" s="31">
-        <f>FIXED(I19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I19*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I19*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D19" s="31">
-        <f>FIXED(J19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J19*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J19*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E19" s="31">
-        <f>FIXED(K19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K19*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K19*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F19" s="31">
-        <f>FIXED(L19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L19*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L19*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G19" s="32">
-        <f>FIXED(M19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M19*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M19*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M19*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M19*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H19" s="1" t="n"/>
@@ -1201,23 +1238,23 @@
         <v/>
       </c>
       <c r="C20" s="31">
-        <f>FIXED(I20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I20*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I20*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D20" s="31">
-        <f>FIXED(J20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J20*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J20*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E20" s="31">
-        <f>FIXED(K20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K20*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K20*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F20" s="31">
-        <f>FIXED(L20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L20*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L20*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G20" s="32">
-        <f>FIXED(M20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M20*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M20*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M20*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M20*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H20" s="1" t="n"/>
@@ -1249,23 +1286,23 @@
         <v/>
       </c>
       <c r="C21" s="31">
-        <f>FIXED(I21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I21*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I21*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D21" s="31">
-        <f>FIXED(J21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J21*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J21*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E21" s="31">
-        <f>FIXED(K21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K21*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K21*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F21" s="31">
-        <f>FIXED(L21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L21*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L21*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G21" s="32">
-        <f>FIXED(M21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M21*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M21*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M21*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M21*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H21" s="1" t="n"/>
@@ -1297,23 +1334,23 @@
         <v/>
       </c>
       <c r="C22" s="31">
-        <f>FIXED(I22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I22*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I22*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D22" s="31">
-        <f>FIXED(J22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J22*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J22*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E22" s="31">
-        <f>FIXED(K22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K22*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K22*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F22" s="31">
-        <f>FIXED(L22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L22*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L22*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G22" s="32">
-        <f>FIXED(M22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M22*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M22*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M22*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M22*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H22" s="1" t="n"/>
@@ -1374,12 +1411,12 @@
       <c r="C25" s="14" t="n"/>
       <c r="D25" s="14" t="n"/>
       <c r="E25" s="14" t="n"/>
-      <c r="F25" s="22" t="inlineStr">
+      <c r="F25" s="40" t="inlineStr">
         <is>
           <t>119 €</t>
         </is>
       </c>
-      <c r="G25" s="23" t="n"/>
+      <c r="G25" s="41" t="n"/>
       <c r="H25" s="1" t="n"/>
       <c r="I25" s="1" t="n"/>
       <c r="J25" s="1" t="n"/>
@@ -1395,11 +1432,11 @@
       <c r="C26" s="24" t="n"/>
       <c r="D26" s="24" t="n"/>
       <c r="E26" s="24" t="n"/>
-      <c r="F26" s="25">
+      <c r="F26" s="42">
         <f>119/3</f>
         <v/>
       </c>
-      <c r="G26" s="26" t="n"/>
+      <c r="G26" s="43" t="n"/>
       <c r="H26" s="1" t="n"/>
       <c r="I26" s="1" t="n"/>
       <c r="J26" s="1" t="n"/>
@@ -1444,23 +1481,23 @@
         <v/>
       </c>
       <c r="C28" s="31">
-        <f>FIXED(I28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I28*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I28*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D28" s="31">
-        <f>FIXED(J28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J28*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J28*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E28" s="31">
-        <f>FIXED(K28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K28*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K28*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F28" s="31">
-        <f>FIXED(L28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L28*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L28*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G28" s="32">
-        <f>FIXED(M28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M28*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M28*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M28*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M28*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H28" s="1" t="n"/>
@@ -1492,23 +1529,23 @@
         <v/>
       </c>
       <c r="C29" s="31">
-        <f>FIXED(I29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I29*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I29*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D29" s="31">
-        <f>FIXED(J29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J29*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J29*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E29" s="31">
-        <f>FIXED(K29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K29*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K29*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F29" s="31">
-        <f>FIXED(L29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L29*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L29*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G29" s="32">
-        <f>FIXED(M29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M29*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M29*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M29*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M29*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H29" s="1" t="n"/>
@@ -1540,23 +1577,23 @@
         <v/>
       </c>
       <c r="C30" s="31">
-        <f>FIXED(I30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I30*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I30*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D30" s="31">
-        <f>FIXED(J30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J30*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J30*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E30" s="31">
-        <f>FIXED(K30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K30*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K30*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F30" s="31">
-        <f>FIXED(L30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L30*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L30*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G30" s="32">
-        <f>FIXED(M30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M30*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M30*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M30*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M30*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H30" s="1" t="n"/>
@@ -1588,23 +1625,23 @@
         <v/>
       </c>
       <c r="C31" s="31">
-        <f>FIXED(I31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I31*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I31*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D31" s="31">
-        <f>FIXED(J31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J31*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J31*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E31" s="31">
-        <f>FIXED(K31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K31*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K31*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F31" s="31">
-        <f>FIXED(L31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L31*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L31*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G31" s="32">
-        <f>FIXED(M31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M31*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M31*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M31*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M31*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H31" s="1" t="n"/>
@@ -1665,12 +1702,12 @@
       <c r="C34" s="14" t="n"/>
       <c r="D34" s="14" t="n"/>
       <c r="E34" s="14" t="n"/>
-      <c r="F34" s="22" t="inlineStr">
+      <c r="F34" s="40" t="inlineStr">
         <is>
           <t>219 €</t>
         </is>
       </c>
-      <c r="G34" s="23" t="n"/>
+      <c r="G34" s="41" t="n"/>
       <c r="H34" s="1" t="n"/>
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="1" t="n"/>
@@ -1686,11 +1723,11 @@
       <c r="C35" s="24" t="n"/>
       <c r="D35" s="24" t="n"/>
       <c r="E35" s="24" t="n"/>
-      <c r="F35" s="25">
+      <c r="F35" s="42">
         <f>219/6</f>
         <v/>
       </c>
-      <c r="G35" s="26" t="n"/>
+      <c r="G35" s="43" t="n"/>
       <c r="H35" s="1" t="n"/>
       <c r="I35" s="1" t="n"/>
       <c r="J35" s="1" t="n"/>
@@ -1735,23 +1772,23 @@
         <v/>
       </c>
       <c r="C37" s="31">
-        <f>FIXED(I37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I37*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I37*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D37" s="31">
-        <f>FIXED(J37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J37*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J37*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E37" s="31">
-        <f>FIXED(K37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K37*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K37*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F37" s="31">
-        <f>FIXED(L37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L37*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L37*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G37" s="32">
-        <f>FIXED(M37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M37*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M37*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M37*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M37*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H37" s="1" t="n"/>
@@ -1783,23 +1820,23 @@
         <v/>
       </c>
       <c r="C38" s="31">
-        <f>FIXED(I38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I38*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I38*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D38" s="31">
-        <f>FIXED(J38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J38*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J38*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E38" s="31">
-        <f>FIXED(K38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K38*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K38*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F38" s="31">
-        <f>FIXED(L38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L38*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L38*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G38" s="32">
-        <f>FIXED(M38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M38*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M38*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M38*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M38*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H38" s="1" t="n"/>
@@ -1831,23 +1868,23 @@
         <v/>
       </c>
       <c r="C39" s="31">
-        <f>FIXED(I39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I39*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I39*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D39" s="31">
-        <f>FIXED(J39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J39*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J39*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E39" s="31">
-        <f>FIXED(K39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K39*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K39*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F39" s="31">
-        <f>FIXED(L39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L39*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L39*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G39" s="32">
-        <f>FIXED(M39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M39*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M39*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M39*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M39*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H39" s="1" t="n"/>
@@ -1879,23 +1916,23 @@
         <v/>
       </c>
       <c r="C40" s="31">
-        <f>FIXED(I40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I40*100,0)&amp;" zo 100"</f>
+        <f>FIXED(I40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(I40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(I40*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="D40" s="31">
-        <f>FIXED(J40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J40*100,0)&amp;" zo 100"</f>
+        <f>FIXED(J40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(J40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(J40*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="E40" s="31">
-        <f>FIXED(K40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K40*100,0)&amp;" zo 100"</f>
+        <f>FIXED(K40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(K40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(K40*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="F40" s="31">
-        <f>FIXED(L40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L40*100,0)&amp;" zo 100"</f>
+        <f>FIXED(L40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(L40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(L40*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="G40" s="32">
-        <f>FIXED(M40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M40*100,0)&amp;" zo 100"</f>
+        <f>FIXED(M40*100,1)&amp;" %"&amp;CHAR(10)&amp;ROUNDUP(M40*$D$8,0)&amp;" z "&amp;$D$8&amp;"  ·  "&amp;ROUNDUP(M40*100,0)&amp;" zo 100 celkovo"</f>
         <v/>
       </c>
       <c r="H40" s="1" t="n"/>

</xml_diff>